<commit_message>
Add shop cultivation survival loop
</commit_message>
<xml_diff>
--- a/docs/GameBalance.xlsx
+++ b/docs/GameBalance.xlsx
@@ -79,9 +79,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ArtifactsTable" displayName="ArtifactsTable" ref="A3:M26" headerRowCount="1">
-  <x:autoFilter ref="A3:M26"/>
-  <x:tableColumns count="13">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ArtifactsTable" displayName="ArtifactsTable" ref="A3:AA32" headerRowCount="1">
+  <x:autoFilter ref="A3:AA32"/>
+  <x:tableColumns count="27">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="名称"/>
     <x:tableColumn id="3" name="体系"/>
@@ -95,14 +95,28 @@
     <x:tableColumn id="11" name="星级3效果"/>
     <x:tableColumn id="12" name="当前状态（测试中/完成）"/>
     <x:tableColumn id="13" name="备注"/>
+    <x:tableColumn id="14" name="summon_base_count"/>
+    <x:tableColumn id="15" name="summon_hp"/>
+    <x:tableColumn id="16" name="summon_attack"/>
+    <x:tableColumn id="17" name="summon_attack_speed"/>
+    <x:tableColumn id="18" name="summon_move_speed"/>
+    <x:tableColumn id="19" name="summon_combat_radius"/>
+    <x:tableColumn id="20" name="summon_return_radius"/>
+    <x:tableColumn id="21" name="summon_respawn_time"/>
+    <x:tableColumn id="22" name="summon_behavior_type"/>
+    <x:tableColumn id="23" name="summon_special_effect"/>
+    <x:tableColumn id="24" name="tier / 品阶"/>
+    <x:tableColumn id="25" name="cost / 价格"/>
+    <x:tableColumn id="26" name="cultivation_requirement"/>
+    <x:tableColumn id="27" name="shop_weight"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SynergiesTable" displayName="SynergiesTable" ref="A3:H18" headerRowCount="1">
-  <x:autoFilter ref="A3:H18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SynergiesTable" displayName="SynergiesTable" ref="A3:H16" headerRowCount="1">
+  <x:autoFilter ref="A3:H16"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="名称"/>
@@ -312,22 +326,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="11.25" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.75" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.75" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.8799991607666" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="9.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.38" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="22.5" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="41.25" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="21.25" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="34" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="14" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="16" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="46" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22.5" customHeight="1">
@@ -380,6 +404,56 @@
       <x:c r="M3" s="6" t="str">
         <x:v>备注</x:v>
       </x:c>
+      <x:c r="N3" s="6" t="str">
+        <x:v>summon_base_count</x:v>
+      </x:c>
+      <x:c r="O3" s="6" t="str">
+        <x:v>summon_hp</x:v>
+      </x:c>
+      <x:c r="P3" s="6" t="str">
+        <x:v>summon_attack</x:v>
+      </x:c>
+      <x:c r="Q3" s="6" t="str">
+        <x:v>summon_attack_speed</x:v>
+      </x:c>
+      <x:c r="R3" s="6" t="str">
+        <x:v>summon_move_speed</x:v>
+      </x:c>
+      <x:c r="S3" s="6" t="str">
+        <x:v>summon_combat_radius</x:v>
+      </x:c>
+      <x:c r="T3" s="6" t="str">
+        <x:v>summon_return_radius</x:v>
+      </x:c>
+      <x:c r="U3" s="6" t="str">
+        <x:v>summon_respawn_time</x:v>
+      </x:c>
+      <x:c r="V3" s="6" t="str">
+        <x:v>summon_behavior_type</x:v>
+      </x:c>
+      <x:c r="W3" s="6" t="str">
+        <x:v>summon_special_effect</x:v>
+      </x:c>
+      <x:c r="X3" t="inlineStr">
+        <x:is>
+          <x:t>tier / 品阶</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y3" t="inlineStr">
+        <x:is>
+          <x:t>cost / 价格</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z3" t="inlineStr">
+        <x:is>
+          <x:t>cultivation_requirement</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AA3" t="inlineStr">
+        <x:is>
+          <x:t>shop_weight</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="6" t="str">
@@ -392,12 +466,12 @@
         <x:v>阵法</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>风</x:v>
+        <x:v>雷</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
         <x:v>formation / aura / attack_speed</x:v>
       </x:c>
-      <x:c r="F4" s="6" t="n">
+      <x:c r="F4" s="6" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str"/>
@@ -405,7 +479,7 @@
         <x:v>半径 125</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
-        <x:v>持续提高玩家法宝攻击速度，并周期性释放小范围风刃脉冲。</x:v>
+        <x:v>持续提高玩家法宝攻击速度，并周期性释放小范围灵刃脉冲。</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
         <x:v>伤害 x1.8；冷却 x0.85</x:v>
@@ -418,6 +492,36 @@
       </x:c>
       <x:c r="M4" s="6" t="str">
         <x:v>攻速 +25%</x:v>
+      </x:c>
+      <x:c r="N4" s="6" t="str"/>
+      <x:c r="O4" s="6" t="str"/>
+      <x:c r="P4" s="6" t="str"/>
+      <x:c r="Q4" s="6" t="str"/>
+      <x:c r="R4" s="6" t="str"/>
+      <x:c r="S4" s="6" t="str"/>
+      <x:c r="T4" s="6" t="str"/>
+      <x:c r="U4" s="6" t="str"/>
+      <x:c r="V4" s="6" t="str"/>
+      <x:c r="W4" s="6" t="str"/>
+      <x:c r="X4" t="inlineStr">
+        <x:is>
+          <x:t>通天灵宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y4" t="inlineStr">
+        <x:is>
+          <x:t>5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z4" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA4" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
@@ -436,10 +540,10 @@
       <x:c r="E5" s="6" t="str">
         <x:v>projectile / projectile</x:v>
       </x:c>
-      <x:c r="F5" s="6" t="n">
+      <x:c r="F5" s="6" t="str">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G5" s="6" t="n">
+      <x:c r="G5" s="6" t="str">
         <x:v>1.35</x:v>
       </x:c>
       <x:c r="H5" s="6" t="str">
@@ -459,6 +563,36 @@
       </x:c>
       <x:c r="M5" s="6" t="str">
         <x:v>穿透 +1；攻击扣血 3，低于 30% 不扣；击杀回复 5</x:v>
+      </x:c>
+      <x:c r="N5" s="6" t="str"/>
+      <x:c r="O5" s="6" t="str"/>
+      <x:c r="P5" s="6" t="str"/>
+      <x:c r="Q5" s="6" t="str"/>
+      <x:c r="R5" s="6" t="str"/>
+      <x:c r="S5" s="6" t="str"/>
+      <x:c r="T5" s="6" t="str"/>
+      <x:c r="U5" s="6" t="str"/>
+      <x:c r="V5" s="6" t="str"/>
+      <x:c r="W5" s="6" t="str"/>
+      <x:c r="X5" t="inlineStr">
+        <x:is>
+          <x:t>通天灵宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y5" t="inlineStr">
+        <x:is>
+          <x:t>5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z5" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA5" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
@@ -477,10 +611,10 @@
       <x:c r="E6" s="6" t="str">
         <x:v>melee / slash</x:v>
       </x:c>
-      <x:c r="F6" s="6" t="n">
+      <x:c r="F6" s="6" t="str">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="G6" s="6" t="n">
+      <x:c r="G6" s="6" t="str">
         <x:v>1.2</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str">
@@ -500,6 +634,36 @@
       </x:c>
       <x:c r="M6" s="6" t="str">
         <x:v>击退 140；攻击扣血 3，低于 30% 不扣；击杀回复 5</x:v>
+      </x:c>
+      <x:c r="N6" s="6" t="str"/>
+      <x:c r="O6" s="6" t="str"/>
+      <x:c r="P6" s="6" t="str"/>
+      <x:c r="Q6" s="6" t="str"/>
+      <x:c r="R6" s="6" t="str"/>
+      <x:c r="S6" s="6" t="str"/>
+      <x:c r="T6" s="6" t="str"/>
+      <x:c r="U6" s="6" t="str"/>
+      <x:c r="V6" s="6" t="str"/>
+      <x:c r="W6" s="6" t="str"/>
+      <x:c r="X6" t="inlineStr">
+        <x:is>
+          <x:t>古宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y6" t="inlineStr">
+        <x:is>
+          <x:t>4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA6" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
@@ -518,10 +682,10 @@
       <x:c r="E7" s="6" t="str">
         <x:v>line_delayed / line</x:v>
       </x:c>
-      <x:c r="F7" s="6" t="n">
+      <x:c r="F7" s="6" t="str">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="G7" s="6" t="n">
+      <x:c r="G7" s="6" t="str">
         <x:v>1.7</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
@@ -540,6 +704,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str"/>
+      <x:c r="N7" s="6" t="str"/>
+      <x:c r="O7" s="6" t="str"/>
+      <x:c r="P7" s="6" t="str"/>
+      <x:c r="Q7" s="6" t="str"/>
+      <x:c r="R7" s="6" t="str"/>
+      <x:c r="S7" s="6" t="str"/>
+      <x:c r="T7" s="6" t="str"/>
+      <x:c r="U7" s="6" t="str"/>
+      <x:c r="V7" s="6" t="str"/>
+      <x:c r="W7" s="6" t="str"/>
+      <x:c r="X7" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y7" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z7" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA7" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="6" t="str">
@@ -557,10 +751,10 @@
       <x:c r="E8" s="6" t="str">
         <x:v>projectile / circle</x:v>
       </x:c>
-      <x:c r="F8" s="6" t="n">
+      <x:c r="F8" s="6" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G8" s="6" t="n">
+      <x:c r="G8" s="6" t="str">
         <x:v>1.3</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
@@ -580,6 +774,36 @@
       </x:c>
       <x:c r="M8" s="6" t="str">
         <x:v>弹射 2</x:v>
+      </x:c>
+      <x:c r="N8" s="6" t="str"/>
+      <x:c r="O8" s="6" t="str"/>
+      <x:c r="P8" s="6" t="str"/>
+      <x:c r="Q8" s="6" t="str"/>
+      <x:c r="R8" s="6" t="str"/>
+      <x:c r="S8" s="6" t="str"/>
+      <x:c r="T8" s="6" t="str"/>
+      <x:c r="U8" s="6" t="str"/>
+      <x:c r="V8" s="6" t="str"/>
+      <x:c r="W8" s="6" t="str"/>
+      <x:c r="X8" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y8" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z8" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA8" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
@@ -598,10 +822,10 @@
       <x:c r="E9" s="6" t="str">
         <x:v>melee / stab</x:v>
       </x:c>
-      <x:c r="F9" s="6" t="n">
+      <x:c r="F9" s="6" t="str">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G9" s="6" t="n">
+      <x:c r="G9" s="6" t="str">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
@@ -620,6 +844,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M9" s="6" t="str"/>
+      <x:c r="N9" s="6" t="str"/>
+      <x:c r="O9" s="6" t="str"/>
+      <x:c r="P9" s="6" t="str"/>
+      <x:c r="Q9" s="6" t="str"/>
+      <x:c r="R9" s="6" t="str"/>
+      <x:c r="S9" s="6" t="str"/>
+      <x:c r="T9" s="6" t="str"/>
+      <x:c r="U9" s="6" t="str"/>
+      <x:c r="V9" s="6" t="str"/>
+      <x:c r="W9" s="6" t="str"/>
+      <x:c r="X9" t="inlineStr">
+        <x:is>
+          <x:t>凡品</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y9" t="inlineStr">
+        <x:is>
+          <x:t>1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z9" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA9" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
       <x:c r="A10" s="6" t="str">
@@ -637,7 +891,7 @@
       <x:c r="E10" s="6" t="str">
         <x:v>formation / aura / damage</x:v>
       </x:c>
-      <x:c r="F10" s="6" t="n">
+      <x:c r="F10" s="6" t="str">
         <x:v>7</x:v>
       </x:c>
       <x:c r="G10" s="6" t="str"/>
@@ -657,6 +911,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M10" s="6" t="str"/>
+      <x:c r="N10" s="6" t="str"/>
+      <x:c r="O10" s="6" t="str"/>
+      <x:c r="P10" s="6" t="str"/>
+      <x:c r="Q10" s="6" t="str"/>
+      <x:c r="R10" s="6" t="str"/>
+      <x:c r="S10" s="6" t="str"/>
+      <x:c r="T10" s="6" t="str"/>
+      <x:c r="U10" s="6" t="str"/>
+      <x:c r="V10" s="6" t="str"/>
+      <x:c r="W10" s="6" t="str"/>
+      <x:c r="X10" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y10" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA10" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="6" t="str">
@@ -674,10 +958,10 @@
       <x:c r="E11" s="6" t="str">
         <x:v>projectile / circle</x:v>
       </x:c>
-      <x:c r="F11" s="6" t="n">
+      <x:c r="F11" s="6" t="str">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="G11" s="6" t="n">
+      <x:c r="G11" s="6" t="str">
         <x:v>1.35</x:v>
       </x:c>
       <x:c r="H11" s="6" t="str">
@@ -697,6 +981,36 @@
       </x:c>
       <x:c r="M11" s="6" t="str">
         <x:v>爆炸半径 60</x:v>
+      </x:c>
+      <x:c r="N11" s="6" t="str"/>
+      <x:c r="O11" s="6" t="str"/>
+      <x:c r="P11" s="6" t="str"/>
+      <x:c r="Q11" s="6" t="str"/>
+      <x:c r="R11" s="6" t="str"/>
+      <x:c r="S11" s="6" t="str"/>
+      <x:c r="T11" s="6" t="str"/>
+      <x:c r="U11" s="6" t="str"/>
+      <x:c r="V11" s="6" t="str"/>
+      <x:c r="W11" s="6" t="str"/>
+      <x:c r="X11" t="inlineStr">
+        <x:is>
+          <x:t>凡品</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y11" t="inlineStr">
+        <x:is>
+          <x:t>1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z11" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA11" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
@@ -715,17 +1029,17 @@
       <x:c r="E12" s="6" t="str">
         <x:v>melee / stab</x:v>
       </x:c>
-      <x:c r="F12" s="6" t="n">
+      <x:c r="F12" s="6" t="str">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G12" s="6" t="n">
+      <x:c r="G12" s="6" t="str">
         <x:v>0.38</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str">
         <x:v>长度 76 / 宽度 32</x:v>
       </x:c>
       <x:c r="I12" s="6" t="str">
-        <x:v>快速近身拳风打击最近敌人，伤害高于远程法宝。</x:v>
+        <x:v>快速近身拳劲打击最近敌人，伤害高于远程法宝。</x:v>
       </x:c>
       <x:c r="J12" s="6" t="str">
         <x:v>伤害 x1.8；冷却 x0.85</x:v>
@@ -738,6 +1052,36 @@
       </x:c>
       <x:c r="M12" s="6" t="str">
         <x:v>击退 120</x:v>
+      </x:c>
+      <x:c r="N12" s="6" t="str"/>
+      <x:c r="O12" s="6" t="str"/>
+      <x:c r="P12" s="6" t="str"/>
+      <x:c r="Q12" s="6" t="str"/>
+      <x:c r="R12" s="6" t="str"/>
+      <x:c r="S12" s="6" t="str"/>
+      <x:c r="T12" s="6" t="str"/>
+      <x:c r="U12" s="6" t="str"/>
+      <x:c r="V12" s="6" t="str"/>
+      <x:c r="W12" s="6" t="str"/>
+      <x:c r="X12" t="inlineStr">
+        <x:is>
+          <x:t>凡品</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y12" t="inlineStr">
+        <x:is>
+          <x:t>1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z12" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA12" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
@@ -756,7 +1100,7 @@
       <x:c r="E13" s="6" t="str">
         <x:v>formation / aura / damage</x:v>
       </x:c>
-      <x:c r="F13" s="6" t="n">
+      <x:c r="F13" s="6" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str"/>
@@ -776,6 +1120,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M13" s="6" t="str"/>
+      <x:c r="N13" s="6" t="str"/>
+      <x:c r="O13" s="6" t="str"/>
+      <x:c r="P13" s="6" t="str"/>
+      <x:c r="Q13" s="6" t="str"/>
+      <x:c r="R13" s="6" t="str"/>
+      <x:c r="S13" s="6" t="str"/>
+      <x:c r="T13" s="6" t="str"/>
+      <x:c r="U13" s="6" t="str"/>
+      <x:c r="V13" s="6" t="str"/>
+      <x:c r="W13" s="6" t="str"/>
+      <x:c r="X13" t="inlineStr">
+        <x:is>
+          <x:t>古宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y13" t="inlineStr">
+        <x:is>
+          <x:t>4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z13" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA13" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
       <x:c r="A14" s="6" t="str">
@@ -793,10 +1167,10 @@
       <x:c r="E14" s="6" t="str">
         <x:v>projectile / projectile</x:v>
       </x:c>
-      <x:c r="F14" s="6" t="n">
+      <x:c r="F14" s="6" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="G14" s="6" t="n">
+      <x:c r="G14" s="6" t="str">
         <x:v>0.95</x:v>
       </x:c>
       <x:c r="H14" s="6" t="str">
@@ -816,6 +1190,36 @@
       </x:c>
       <x:c r="M14" s="6" t="str">
         <x:v>穿透 +1</x:v>
+      </x:c>
+      <x:c r="N14" s="6" t="str"/>
+      <x:c r="O14" s="6" t="str"/>
+      <x:c r="P14" s="6" t="str"/>
+      <x:c r="Q14" s="6" t="str"/>
+      <x:c r="R14" s="6" t="str"/>
+      <x:c r="S14" s="6" t="str"/>
+      <x:c r="T14" s="6" t="str"/>
+      <x:c r="U14" s="6" t="str"/>
+      <x:c r="V14" s="6" t="str"/>
+      <x:c r="W14" s="6" t="str"/>
+      <x:c r="X14" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y14" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z14" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA14" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
@@ -854,6 +1258,36 @@
       <x:c r="M15" s="6" t="str">
         <x:v>护盾 12，上限 36</x:v>
       </x:c>
+      <x:c r="N15" s="6" t="str"/>
+      <x:c r="O15" s="6" t="str"/>
+      <x:c r="P15" s="6" t="str"/>
+      <x:c r="Q15" s="6" t="str"/>
+      <x:c r="R15" s="6" t="str"/>
+      <x:c r="S15" s="6" t="str"/>
+      <x:c r="T15" s="6" t="str"/>
+      <x:c r="U15" s="6" t="str"/>
+      <x:c r="V15" s="6" t="str"/>
+      <x:c r="W15" s="6" t="str"/>
+      <x:c r="X15" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y15" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z15" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA15" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
       <x:c r="A16" s="6" t="str">
@@ -871,10 +1305,10 @@
       <x:c r="E16" s="6" t="str">
         <x:v>orbit</x:v>
       </x:c>
-      <x:c r="F16" s="6" t="n">
+      <x:c r="F16" s="6" t="str">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G16" s="6" t="n">
+      <x:c r="G16" s="6" t="str">
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="H16" s="6" t="str">
@@ -893,6 +1327,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M16" s="6" t="str"/>
+      <x:c r="N16" s="6" t="str"/>
+      <x:c r="O16" s="6" t="str"/>
+      <x:c r="P16" s="6" t="str"/>
+      <x:c r="Q16" s="6" t="str"/>
+      <x:c r="R16" s="6" t="str"/>
+      <x:c r="S16" s="6" t="str"/>
+      <x:c r="T16" s="6" t="str"/>
+      <x:c r="U16" s="6" t="str"/>
+      <x:c r="V16" s="6" t="str"/>
+      <x:c r="W16" s="6" t="str"/>
+      <x:c r="X16" t="inlineStr">
+        <x:is>
+          <x:t>古宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y16" t="inlineStr">
+        <x:is>
+          <x:t>4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z16" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA16" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="17" ht="36" customHeight="1">
       <x:c r="A17" s="6" t="str">
@@ -905,15 +1369,15 @@
         <x:v>法修</x:v>
       </x:c>
       <x:c r="D17" s="6" t="str">
-        <x:v>风</x:v>
+        <x:v>木</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
         <x:v>projectile / circle</x:v>
       </x:c>
-      <x:c r="F17" s="6" t="n">
+      <x:c r="F17" s="6" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G17" s="6" t="n">
+      <x:c r="G17" s="6" t="str">
         <x:v>1.15</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str">
@@ -932,6 +1396,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M17" s="6" t="str"/>
+      <x:c r="N17" s="6" t="str"/>
+      <x:c r="O17" s="6" t="str"/>
+      <x:c r="P17" s="6" t="str"/>
+      <x:c r="Q17" s="6" t="str"/>
+      <x:c r="R17" s="6" t="str"/>
+      <x:c r="S17" s="6" t="str"/>
+      <x:c r="T17" s="6" t="str"/>
+      <x:c r="U17" s="6" t="str"/>
+      <x:c r="V17" s="6" t="str"/>
+      <x:c r="W17" s="6" t="str"/>
+      <x:c r="X17" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y17" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z17" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA17" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
       <x:c r="A18" s="6" t="str">
@@ -949,7 +1443,7 @@
       <x:c r="E18" s="6" t="str">
         <x:v>formation / aura / heal</x:v>
       </x:c>
-      <x:c r="F18" s="6" t="n">
+      <x:c r="F18" s="6" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G18" s="6" t="str"/>
@@ -971,6 +1465,36 @@
       <x:c r="M18" s="6" t="str">
         <x:v>治疗 3</x:v>
       </x:c>
+      <x:c r="N18" s="6" t="str"/>
+      <x:c r="O18" s="6" t="str"/>
+      <x:c r="P18" s="6" t="str"/>
+      <x:c r="Q18" s="6" t="str"/>
+      <x:c r="R18" s="6" t="str"/>
+      <x:c r="S18" s="6" t="str"/>
+      <x:c r="T18" s="6" t="str"/>
+      <x:c r="U18" s="6" t="str"/>
+      <x:c r="V18" s="6" t="str"/>
+      <x:c r="W18" s="6" t="str"/>
+      <x:c r="X18" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y18" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z18" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA18" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="19" ht="36" customHeight="1">
       <x:c r="A19" s="6" t="str">
@@ -988,10 +1512,10 @@
       <x:c r="E19" s="6" t="str">
         <x:v>beam / beam</x:v>
       </x:c>
-      <x:c r="F19" s="6" t="n">
+      <x:c r="F19" s="6" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G19" s="6" t="n">
+      <x:c r="G19" s="6" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str">
@@ -1010,6 +1534,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M19" s="6" t="str"/>
+      <x:c r="N19" s="6" t="str"/>
+      <x:c r="O19" s="6" t="str"/>
+      <x:c r="P19" s="6" t="str"/>
+      <x:c r="Q19" s="6" t="str"/>
+      <x:c r="R19" s="6" t="str"/>
+      <x:c r="S19" s="6" t="str"/>
+      <x:c r="T19" s="6" t="str"/>
+      <x:c r="U19" s="6" t="str"/>
+      <x:c r="V19" s="6" t="str"/>
+      <x:c r="W19" s="6" t="str"/>
+      <x:c r="X19" t="inlineStr">
+        <x:is>
+          <x:t>通天灵宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y19" t="inlineStr">
+        <x:is>
+          <x:t>5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z19" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA19" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
       <x:c r="A20" s="6" t="str">
@@ -1027,29 +1581,59 @@
       <x:c r="E20" s="6" t="str">
         <x:v>melee / circle</x:v>
       </x:c>
-      <x:c r="F20" s="6" t="n">
+      <x:c r="F20" s="6" t="str">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="G20" s="6" t="n">
+      <x:c r="G20" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H20" s="6" t="str">
         <x:v>半径 98</x:v>
       </x:c>
       <x:c r="I20" s="6" t="str">
-        <x:v>贴身旋风扫腿，对周围一圈敌人造成较高伤害并轻微击退。</x:v>
+        <x:v>贴身旋身扫腿，对周围一圈敌人造成较高伤害并轻微击退。</x:v>
       </x:c>
       <x:c r="J20" s="6" t="str">
         <x:v>伤害 x1.8；冷却 x0.85</x:v>
       </x:c>
       <x:c r="K20" s="6" t="str">
-        <x:v>伤害 x3.0；冷却 x0.7；旋风腿范围 +50%</x:v>
+        <x:v>伤害 x3.0；冷却 x0.7；旋身腿范围 +50%</x:v>
       </x:c>
       <x:c r="L20" s="6" t="str">
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M20" s="6" t="str">
         <x:v>击退 90</x:v>
+      </x:c>
+      <x:c r="N20" s="6" t="str"/>
+      <x:c r="O20" s="6" t="str"/>
+      <x:c r="P20" s="6" t="str"/>
+      <x:c r="Q20" s="6" t="str"/>
+      <x:c r="R20" s="6" t="str"/>
+      <x:c r="S20" s="6" t="str"/>
+      <x:c r="T20" s="6" t="str"/>
+      <x:c r="U20" s="6" t="str"/>
+      <x:c r="V20" s="6" t="str"/>
+      <x:c r="W20" s="6" t="str"/>
+      <x:c r="X20" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y20" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z20" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA20" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
@@ -1063,15 +1647,15 @@
         <x:v>剑修</x:v>
       </x:c>
       <x:c r="D21" s="6" t="str">
-        <x:v>风</x:v>
+        <x:v>金</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
         <x:v>melee / stab</x:v>
       </x:c>
-      <x:c r="F21" s="6" t="n">
+      <x:c r="F21" s="6" t="str">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="G21" s="6" t="n">
+      <x:c r="G21" s="6" t="str">
         <x:v>1.05</x:v>
       </x:c>
       <x:c r="H21" s="6" t="str">
@@ -1090,6 +1674,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M21" s="6" t="str"/>
+      <x:c r="N21" s="6" t="str"/>
+      <x:c r="O21" s="6" t="str"/>
+      <x:c r="P21" s="6" t="str"/>
+      <x:c r="Q21" s="6" t="str"/>
+      <x:c r="R21" s="6" t="str"/>
+      <x:c r="S21" s="6" t="str"/>
+      <x:c r="T21" s="6" t="str"/>
+      <x:c r="U21" s="6" t="str"/>
+      <x:c r="V21" s="6" t="str"/>
+      <x:c r="W21" s="6" t="str"/>
+      <x:c r="X21" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y21" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z21" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA21" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="22" ht="36" customHeight="1">
       <x:c r="A22" s="6" t="str">
@@ -1107,10 +1721,10 @@
       <x:c r="E22" s="6" t="str">
         <x:v>projectile / circle</x:v>
       </x:c>
-      <x:c r="F22" s="6" t="n">
+      <x:c r="F22" s="6" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G22" s="6" t="n">
+      <x:c r="G22" s="6" t="str">
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="H22" s="6" t="str">
@@ -1130,6 +1744,36 @@
       </x:c>
       <x:c r="M22" s="6" t="str">
         <x:v>穿透 +3</x:v>
+      </x:c>
+      <x:c r="N22" s="6" t="str"/>
+      <x:c r="O22" s="6" t="str"/>
+      <x:c r="P22" s="6" t="str"/>
+      <x:c r="Q22" s="6" t="str"/>
+      <x:c r="R22" s="6" t="str"/>
+      <x:c r="S22" s="6" t="str"/>
+      <x:c r="T22" s="6" t="str"/>
+      <x:c r="U22" s="6" t="str"/>
+      <x:c r="V22" s="6" t="str"/>
+      <x:c r="W22" s="6" t="str"/>
+      <x:c r="X22" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y22" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z22" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA22" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
@@ -1148,10 +1792,10 @@
       <x:c r="E23" s="6" t="str">
         <x:v>melee / slash</x:v>
       </x:c>
-      <x:c r="F23" s="6" t="n">
+      <x:c r="F23" s="6" t="str">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="G23" s="6" t="n">
+      <x:c r="G23" s="6" t="str">
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="H23" s="6" t="str">
@@ -1170,6 +1814,36 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M23" s="6" t="str"/>
+      <x:c r="N23" s="6" t="str"/>
+      <x:c r="O23" s="6" t="str"/>
+      <x:c r="P23" s="6" t="str"/>
+      <x:c r="Q23" s="6" t="str"/>
+      <x:c r="R23" s="6" t="str"/>
+      <x:c r="S23" s="6" t="str"/>
+      <x:c r="T23" s="6" t="str"/>
+      <x:c r="U23" s="6" t="str"/>
+      <x:c r="V23" s="6" t="str"/>
+      <x:c r="W23" s="6" t="str"/>
+      <x:c r="X23" t="inlineStr">
+        <x:is>
+          <x:t>凡品</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y23" t="inlineStr">
+        <x:is>
+          <x:t>1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z23" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA23" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
       <x:c r="A24" s="6" t="str">
@@ -1187,29 +1861,59 @@
       <x:c r="E24" s="6" t="str">
         <x:v>melee / slash</x:v>
       </x:c>
-      <x:c r="F24" s="6" t="n">
+      <x:c r="F24" s="6" t="str">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="G24" s="6" t="n">
+      <x:c r="G24" s="6" t="str">
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="H24" s="6" t="str">
         <x:v>长度 112 / 宽度 110</x:v>
       </x:c>
       <x:c r="I24" s="6" t="str">
-        <x:v>挥出爆发掌风打击前方扇形敌人，并将敌人击退。</x:v>
+        <x:v>挥出爆发掌劲打击前方扇形敌人，并将敌人击退。</x:v>
       </x:c>
       <x:c r="J24" s="6" t="str">
         <x:v>伤害 x1.8；冷却 x0.85</x:v>
       </x:c>
       <x:c r="K24" s="6" t="str">
-        <x:v>伤害 x3.0；冷却 x0.7；掌风角度 +50%</x:v>
+        <x:v>伤害 x3.0；冷却 x0.7；掌劲角度 +50%</x:v>
       </x:c>
       <x:c r="L24" s="6" t="str">
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="M24" s="6" t="str">
         <x:v>击退 360</x:v>
+      </x:c>
+      <x:c r="N24" s="6" t="str"/>
+      <x:c r="O24" s="6" t="str"/>
+      <x:c r="P24" s="6" t="str"/>
+      <x:c r="Q24" s="6" t="str"/>
+      <x:c r="R24" s="6" t="str"/>
+      <x:c r="S24" s="6" t="str"/>
+      <x:c r="T24" s="6" t="str"/>
+      <x:c r="U24" s="6" t="str"/>
+      <x:c r="V24" s="6" t="str"/>
+      <x:c r="W24" s="6" t="str"/>
+      <x:c r="X24" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y24" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z24" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA24" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="25" ht="36" customHeight="1">
@@ -1228,10 +1932,10 @@
       <x:c r="E25" s="6" t="str">
         <x:v>projectile / projectile</x:v>
       </x:c>
-      <x:c r="F25" s="6" t="n">
+      <x:c r="F25" s="6" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G25" s="6" t="n">
+      <x:c r="G25" s="6" t="str">
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="H25" s="6" t="str">
@@ -1251,6 +1955,36 @@
       </x:c>
       <x:c r="M25" s="6" t="str">
         <x:v>中毒 3/秒，3秒</x:v>
+      </x:c>
+      <x:c r="N25" s="6" t="str"/>
+      <x:c r="O25" s="6" t="str"/>
+      <x:c r="P25" s="6" t="str"/>
+      <x:c r="Q25" s="6" t="str"/>
+      <x:c r="R25" s="6" t="str"/>
+      <x:c r="S25" s="6" t="str"/>
+      <x:c r="T25" s="6" t="str"/>
+      <x:c r="U25" s="6" t="str"/>
+      <x:c r="V25" s="6" t="str"/>
+      <x:c r="W25" s="6" t="str"/>
+      <x:c r="X25" t="inlineStr">
+        <x:is>
+          <x:t>古宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y25" t="inlineStr">
+        <x:is>
+          <x:t>4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z25" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA25" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="26" ht="36" customHeight="1">
@@ -1269,7 +2003,7 @@
       <x:c r="E26" s="6" t="str">
         <x:v>formation / aura / slow</x:v>
       </x:c>
-      <x:c r="F26" s="6" t="n">
+      <x:c r="F26" s="6" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G26" s="6" t="str"/>
@@ -1291,15 +2025,591 @@
       <x:c r="M26" s="6" t="str">
         <x:v>减速 35%</x:v>
       </x:c>
+      <x:c r="N26" s="6" t="str"/>
+      <x:c r="O26" s="6" t="str"/>
+      <x:c r="P26" s="6" t="str"/>
+      <x:c r="Q26" s="6" t="str"/>
+      <x:c r="R26" s="6" t="str"/>
+      <x:c r="S26" s="6" t="str"/>
+      <x:c r="T26" s="6" t="str"/>
+      <x:c r="U26" s="6" t="str"/>
+      <x:c r="V26" s="6" t="str"/>
+      <x:c r="W26" s="6" t="str"/>
+      <x:c r="X26" t="inlineStr">
+        <x:is>
+          <x:t>凡品</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y26" t="inlineStr">
+        <x:is>
+          <x:t>1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z26" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA26" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="36" customHeight="1">
+      <x:c r="A27" s="6" t="str">
+        <x:v>sword_puppet</x:v>
+      </x:c>
+      <x:c r="B27" s="6" t="str">
+        <x:v>剑傀儡</x:v>
+      </x:c>
+      <x:c r="C27" s="6" t="str">
+        <x:v>召唤</x:v>
+      </x:c>
+      <x:c r="D27" s="6" t="str">
+        <x:v>金</x:v>
+      </x:c>
+      <x:c r="E27" s="6" t="str">
+        <x:v>summon / slash / melee</x:v>
+      </x:c>
+      <x:c r="F27" s="6" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G27" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H27" s="6" t="str">
+        <x:v>combat 500 / return 700</x:v>
+      </x:c>
+      <x:c r="I27" s="6" t="str">
+        <x:v>基础数量1；生命100；攻击15；攻速1.0；近战扇形挥砍；6秒重生</x:v>
+      </x:c>
+      <x:c r="J27" s="6" t="str">
+        <x:v>生命+50%；攻击+50%</x:v>
+      </x:c>
+      <x:c r="K27" s="6" t="str">
+        <x:v>攻击范围+30%；每第三次攻击造成200%伤害</x:v>
+      </x:c>
+      <x:c r="L27" s="6" t="str">
+        <x:v>测试中</x:v>
+      </x:c>
+      <x:c r="M27" s="6" t="str">
+        <x:v>近战主力输出</x:v>
+      </x:c>
+      <x:c r="N27" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O27" s="6" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P27" s="6" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="Q27" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R27" s="6" t="n">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="S27" s="6" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="T27" s="6" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="U27" s="6" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V27" s="6" t="str">
+        <x:v>melee</x:v>
+      </x:c>
+      <x:c r="W27" s="6" t="str">
+        <x:v>追击最近敌人，近战扇形挥砍</x:v>
+      </x:c>
+      <x:c r="X27" t="inlineStr">
+        <x:is>
+          <x:t>凡品</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y27" t="inlineStr">
+        <x:is>
+          <x:t>1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z27" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA27" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="36" customHeight="1">
+      <x:c r="A28" s="6" t="str">
+        <x:v>crossbow_puppet</x:v>
+      </x:c>
+      <x:c r="B28" s="6" t="str">
+        <x:v>弩傀儡</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="str">
+        <x:v>召唤</x:v>
+      </x:c>
+      <x:c r="D28" s="6" t="str">
+        <x:v>雷</x:v>
+      </x:c>
+      <x:c r="E28" s="6" t="str">
+        <x:v>summon / projectile / ranged</x:v>
+      </x:c>
+      <x:c r="F28" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G28" s="6" t="n">
+        <x:v>0.67</x:v>
+      </x:c>
+      <x:c r="H28" s="6" t="str">
+        <x:v>combat 600 / return 700</x:v>
+      </x:c>
+      <x:c r="I28" s="6" t="str">
+        <x:v>基础数量1；生命70；攻击10；攻速1.5；保持距离发射灵能箭；6秒重生</x:v>
+      </x:c>
+      <x:c r="J28" s="6" t="str">
+        <x:v>攻击+50%；攻速+30%</x:v>
+      </x:c>
+      <x:c r="K28" s="6" t="str">
+        <x:v>灵能箭弹射1次</x:v>
+      </x:c>
+      <x:c r="L28" s="6" t="str">
+        <x:v>测试中</x:v>
+      </x:c>
+      <x:c r="M28" s="6" t="str">
+        <x:v>后排持续输出</x:v>
+      </x:c>
+      <x:c r="N28" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O28" s="6" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="P28" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q28" s="6" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="R28" s="6" t="n">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="S28" s="6" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="T28" s="6" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="U28" s="6" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V28" s="6" t="str">
+        <x:v>ranged</x:v>
+      </x:c>
+      <x:c r="W28" s="6" t="str">
+        <x:v>保持距离，优先攻击最近敌人</x:v>
+      </x:c>
+      <x:c r="X28" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y28" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z28" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA28" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="36" customHeight="1">
+      <x:c r="A29" s="6" t="str">
+        <x:v>iron_guard_puppet</x:v>
+      </x:c>
+      <x:c r="B29" s="6" t="str">
+        <x:v>铁卫傀儡</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="str">
+        <x:v>召唤</x:v>
+      </x:c>
+      <x:c r="D29" s="6" t="str">
+        <x:v>土</x:v>
+      </x:c>
+      <x:c r="E29" s="6" t="str">
+        <x:v>summon / melee / tank</x:v>
+      </x:c>
+      <x:c r="F29" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G29" s="6" t="n">
+        <x:v>1.43</x:v>
+      </x:c>
+      <x:c r="H29" s="6" t="str">
+        <x:v>combat 450 / return 600</x:v>
+      </x:c>
+      <x:c r="I29" s="6" t="str">
+        <x:v>基础数量1；生命300；攻击8；攻速0.7；每5秒嘲讽半径300内敌人2秒；8秒重生</x:v>
+      </x:c>
+      <x:c r="J29" s="6" t="str">
+        <x:v>生命+80%</x:v>
+      </x:c>
+      <x:c r="K29" s="6" t="str">
+        <x:v>嘲讽范围+50%；受到攻击时释放震荡波</x:v>
+      </x:c>
+      <x:c r="L29" s="6" t="str">
+        <x:v>测试中</x:v>
+      </x:c>
+      <x:c r="M29" s="6" t="str">
+        <x:v>尽量站在玩家与怪群之间</x:v>
+      </x:c>
+      <x:c r="N29" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O29" s="6" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="P29" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q29" s="6" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="R29" s="6" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="S29" s="6" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="T29" s="6" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="U29" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="V29" s="6" t="str">
+        <x:v>tank</x:v>
+      </x:c>
+      <x:c r="W29" s="6" t="str">
+        <x:v>5秒嘲讽；阻挡怪群</x:v>
+      </x:c>
+      <x:c r="X29" t="inlineStr">
+        <x:is>
+          <x:t>古宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y29" t="inlineStr">
+        <x:is>
+          <x:t>4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z29" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA29" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="36" customHeight="1">
+      <x:c r="A30" s="6" t="str">
+        <x:v>turret</x:v>
+      </x:c>
+      <x:c r="B30" s="6" t="str">
+        <x:v>炮台</x:v>
+      </x:c>
+      <x:c r="C30" s="6" t="str">
+        <x:v>召唤</x:v>
+      </x:c>
+      <x:c r="D30" s="6" t="str">
+        <x:v>火</x:v>
+      </x:c>
+      <x:c r="E30" s="6" t="str">
+        <x:v>summon / projectile / turret</x:v>
+      </x:c>
+      <x:c r="F30" s="6" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G30" s="6" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="H30" s="6" t="str">
+        <x:v>combat 700 / redeploy 900</x:v>
+      </x:c>
+      <x:c r="I30" s="6" t="str">
+        <x:v>基础数量1；生命120；攻击18；攻速0.8；固定炮台发射小范围爆炸炮弹；10秒重生</x:v>
+      </x:c>
+      <x:c r="J30" s="6" t="str">
+        <x:v>攻击+50%</x:v>
+      </x:c>
+      <x:c r="K30" s="6" t="str">
+        <x:v>爆炸范围+50%</x:v>
+      </x:c>
+      <x:c r="L30" s="6" t="str">
+        <x:v>测试中</x:v>
+      </x:c>
+      <x:c r="M30" s="6" t="str">
+        <x:v>玩家距离超过900时，2秒后在玩家附近重新建造</x:v>
+      </x:c>
+      <x:c r="N30" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O30" s="6" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="P30" s="6" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="Q30" s="6" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="R30" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S30" s="6" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="T30" s="6" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="U30" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V30" s="6" t="str">
+        <x:v>turret</x:v>
+      </x:c>
+      <x:c r="W30" s="6" t="str">
+        <x:v>固定不移动，超距重新部署</x:v>
+      </x:c>
+      <x:c r="X30" t="inlineStr">
+        <x:is>
+          <x:t>法器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y30" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z30" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA30" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="36" customHeight="1">
+      <x:c r="A31" s="6" t="str">
+        <x:v>ghost</x:v>
+      </x:c>
+      <x:c r="B31" s="6" t="str">
+        <x:v>幽魂</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="str">
+        <x:v>召唤</x:v>
+      </x:c>
+      <x:c r="D31" s="6" t="str">
+        <x:v>水</x:v>
+      </x:c>
+      <x:c r="E31" s="6" t="str">
+        <x:v>summon / line / ghost</x:v>
+      </x:c>
+      <x:c r="F31" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G31" s="6" t="n">
+        <x:v>0.83</x:v>
+      </x:c>
+      <x:c r="H31" s="6" t="str">
+        <x:v>combat 700 / return 900</x:v>
+      </x:c>
+      <x:c r="I31" s="6" t="str">
+        <x:v>基础数量2；生命60；攻击8；攻速1.2；穿过敌人造成伤害并回复玩家生命；4秒重生</x:v>
+      </x:c>
+      <x:c r="J31" s="6" t="str">
+        <x:v>攻击+50%；回复量+50%</x:v>
+      </x:c>
+      <x:c r="K31" s="6" t="str">
+        <x:v>命中触发灵魂冲击</x:v>
+      </x:c>
+      <x:c r="L31" s="6" t="str">
+        <x:v>测试中</x:v>
+      </x:c>
+      <x:c r="M31" s="6" t="str">
+        <x:v>机动骚扰，无实体阻挡</x:v>
+      </x:c>
+      <x:c r="N31" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O31" s="6" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="P31" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q31" s="6" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="R31" s="6" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="S31" s="6" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="T31" s="6" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="U31" s="6" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="V31" s="6" t="str">
+        <x:v>ghost</x:v>
+      </x:c>
+      <x:c r="W31" s="6" t="str">
+        <x:v>穿透冲刺，命中回血</x:v>
+      </x:c>
+      <x:c r="X31" t="inlineStr">
+        <x:is>
+          <x:t>灵器</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y31" t="inlineStr">
+        <x:is>
+          <x:t>3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z31" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA31" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="36" customHeight="1">
+      <x:c r="A32" s="6" t="str">
+        <x:v>poison_bug</x:v>
+      </x:c>
+      <x:c r="B32" s="6" t="str">
+        <x:v>毒虫</x:v>
+      </x:c>
+      <x:c r="C32" s="6" t="str">
+        <x:v>召唤</x:v>
+      </x:c>
+      <x:c r="D32" s="6" t="str">
+        <x:v>毒</x:v>
+      </x:c>
+      <x:c r="E32" s="6" t="str">
+        <x:v>summon / melee / swarm</x:v>
+      </x:c>
+      <x:c r="F32" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G32" s="6" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H32" s="6" t="str">
+        <x:v>combat 450 / return 650</x:v>
+      </x:c>
+      <x:c r="I32" s="6" t="str">
+        <x:v>基础数量3；生命30；攻击5；攻速2.0；近战撕咬附加中毒；3秒重生</x:v>
+      </x:c>
+      <x:c r="J32" s="6" t="str">
+        <x:v>数量+1；攻击+50%</x:v>
+      </x:c>
+      <x:c r="K32" s="6" t="str">
+        <x:v>中毒伤害翻倍</x:v>
+      </x:c>
+      <x:c r="L32" s="6" t="str">
+        <x:v>测试中</x:v>
+      </x:c>
+      <x:c r="M32" s="6" t="str">
+        <x:v>敌人死亡20%概率补充毒虫，总数不超过上限</x:v>
+      </x:c>
+      <x:c r="N32" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O32" s="6" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="P32" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="Q32" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R32" s="6" t="n">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="S32" s="6" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="T32" s="6" t="n">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="U32" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="V32" s="6" t="str">
+        <x:v>swarm</x:v>
+      </x:c>
+      <x:c r="W32" s="6" t="str">
+        <x:v>轻量寻路，过远回防或瞬移</x:v>
+      </x:c>
+      <x:c r="X32" t="inlineStr">
+        <x:is>
+          <x:t>通天灵宝</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y32" t="inlineStr">
+        <x:is>
+          <x:t>5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Z32" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="AA32" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A2:M2"/>
+    <x:mergeCell ref="A1:W1"/>
+    <x:mergeCell ref="A2:W2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra36a99d7160a4039"/>
+    <x:tablePart ns1:id="Ra36a99d7160a4039"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1308,14 +2618,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="38.75" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="38.75" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="31.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="37.5" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22.5" customHeight="1">
@@ -1465,15 +2775,19 @@
         <x:v>体系</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
-        <x:v>召唤流预留羁绊</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="str"/>
-      <x:c r="F8" s="6" t="str"/>
+        <x:v>所有召唤法宝：数量上限 +1</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>所有召唤法宝：数量上限额外 +1；重生时间 -50%</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>所有召唤法宝：数量上限额外 +2；召唤物死亡释放灵力冲击</x:v>
+      </x:c>
       <x:c r="G8" s="6" t="str">
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
-        <x:v>UI 已显示；召唤玩法仍为验证/预留方向</x:v>
+        <x:v>已实现：summon_extra_count / summon_respawn_time_multiplier / summon_death_burst_enabled</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
@@ -1524,16 +2838,16 @@
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="6" t="str">
-        <x:v>wind</x:v>
+        <x:v>poison</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>风</x:v>
+        <x:v>毒</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
         <x:v>属性</x:v>
       </x:c>
       <x:c r="D11" s="6" t="str">
-        <x:v>阈值3：属性羁绊预留：风属性 Build 方向</x:v>
+        <x:v>阈值3：属性羁绊预留：毒属性 Build 方向</x:v>
       </x:c>
       <x:c r="E11" s="6" t="str"/>
       <x:c r="F11" s="6" t="str"/>
@@ -1546,16 +2860,16 @@
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
       <x:c r="A12" s="6" t="str">
-        <x:v>poison</x:v>
+        <x:v>thunder</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>毒</x:v>
+        <x:v>雷</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
         <x:v>属性</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:v>阈值3：属性羁绊预留：毒属性 Build 方向</x:v>
+        <x:v>阈值2：属性羁绊预留：雷属性 Build 方向</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str"/>
       <x:c r="F12" s="6" t="str"/>
@@ -1568,16 +2882,16 @@
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
       <x:c r="A13" s="6" t="str">
-        <x:v>thunder</x:v>
+        <x:v>water</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
-        <x:v>雷</x:v>
+        <x:v>水</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
         <x:v>属性</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
-        <x:v>阈值2：属性羁绊预留：雷属性 Build 方向</x:v>
+        <x:v>阈值2：属性羁绊预留：水属性 Build 方向</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str"/>
       <x:c r="F13" s="6" t="str"/>
@@ -1590,16 +2904,16 @@
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
       <x:c r="A14" s="6" t="str">
-        <x:v>water</x:v>
+        <x:v>earth</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
-        <x:v>水</x:v>
+        <x:v>土</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
         <x:v>属性</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>阈值2：属性羁绊预留：水属性 Build 方向</x:v>
+        <x:v>阈值2：属性羁绊预留：土属性 Build 方向</x:v>
       </x:c>
       <x:c r="E14" s="6" t="str"/>
       <x:c r="F14" s="6" t="str"/>
@@ -1612,16 +2926,16 @@
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>earth</x:v>
+        <x:v>metal</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
-        <x:v>土</x:v>
+        <x:v>金</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
         <x:v>属性</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
-        <x:v>阈值2：属性羁绊预留：土属性 Build 方向</x:v>
+        <x:v>阈值2：属性羁绊预留：金属性 Build 方向</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str"/>
       <x:c r="F15" s="6" t="str"/>
@@ -1634,16 +2948,16 @@
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
       <x:c r="A16" s="6" t="str">
-        <x:v>metal</x:v>
+        <x:v>wood</x:v>
       </x:c>
       <x:c r="B16" s="6" t="str">
-        <x:v>金</x:v>
+        <x:v>木</x:v>
       </x:c>
       <x:c r="C16" s="6" t="str">
         <x:v>属性</x:v>
       </x:c>
       <x:c r="D16" s="6" t="str">
-        <x:v>阈值2：属性羁绊预留：金属性 Build 方向</x:v>
+        <x:v>阈值2：属性羁绊预留：木属性 Build 方向</x:v>
       </x:c>
       <x:c r="E16" s="6" t="str"/>
       <x:c r="F16" s="6" t="str"/>
@@ -1651,50 +2965,6 @@
         <x:v>测试中</x:v>
       </x:c>
       <x:c r="H16" s="6" t="str">
-        <x:v>当前仅显示进度与提示，未实现战斗效果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="36" customHeight="1">
-      <x:c r="A17" s="6" t="str">
-        <x:v>wood</x:v>
-      </x:c>
-      <x:c r="B17" s="6" t="str">
-        <x:v>木</x:v>
-      </x:c>
-      <x:c r="C17" s="6" t="str">
-        <x:v>属性</x:v>
-      </x:c>
-      <x:c r="D17" s="6" t="str">
-        <x:v>阈值2：属性羁绊预留：木属性 Build 方向</x:v>
-      </x:c>
-      <x:c r="E17" s="6" t="str"/>
-      <x:c r="F17" s="6" t="str"/>
-      <x:c r="G17" s="6" t="str">
-        <x:v>测试中</x:v>
-      </x:c>
-      <x:c r="H17" s="6" t="str">
-        <x:v>当前仅显示进度与提示，未实现战斗效果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="36" customHeight="1">
-      <x:c r="A18" s="6" t="str">
-        <x:v>dark</x:v>
-      </x:c>
-      <x:c r="B18" s="6" t="str">
-        <x:v>暗</x:v>
-      </x:c>
-      <x:c r="C18" s="6" t="str">
-        <x:v>属性</x:v>
-      </x:c>
-      <x:c r="D18" s="6" t="str">
-        <x:v>阈值2：属性羁绊预留：暗属性 Build 方向</x:v>
-      </x:c>
-      <x:c r="E18" s="6" t="str"/>
-      <x:c r="F18" s="6" t="str"/>
-      <x:c r="G18" s="6" t="str">
-        <x:v>测试中</x:v>
-      </x:c>
-      <x:c r="H18" s="6" t="str">
         <x:v>当前仅显示进度与提示，未实现战斗效果</x:v>
       </x:c>
     </x:row>
@@ -1705,7 +2975,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfda46139e4094005"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafa84f5115a14823"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>